<commit_message>
Update demo outputs and regenerate cross-package artifacts
</commit_message>
<xml_diff>
--- a/iivw/demo/iivw_results.xlsx
+++ b/iivw/demo/iivw_results.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="72" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="144" uniqueCount="33">
   <si>
     <t>IIW vs FIPTIW: Cognitive Score</t>
   </si>
@@ -118,10 +118,1468 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="338">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
+  <fonts count="675">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1590,7 +3048,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="253">
+  <borders count="505">
     <border>
       <left/>
       <right/>
@@ -3314,11 +4772,1727 @@
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="253">
+  <cellXfs count="505">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -4301,6 +7475,990 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="337" fillId="0" borderId="252" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="253" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="254" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="255" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="256" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="257" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="258" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="259" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="260" xfId="0"/>
+    <xf numFmtId="0" fontId="338" fillId="0" borderId="261" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="339" fillId="0" borderId="262" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="340" fillId="0" borderId="263" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="341" fillId="0" borderId="264" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="342" fillId="0" borderId="265" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="343" fillId="0" borderId="266" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="345" fillId="0" borderId="267" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="347" fillId="0" borderId="268" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="349" fillId="0" borderId="269" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="350" fillId="0" borderId="270" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="351" fillId="0" borderId="271" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="352" fillId="0" borderId="272" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="353" fillId="0" borderId="273" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="354" fillId="0" borderId="274" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="355" fillId="0" borderId="275" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="356" fillId="0" borderId="276" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="357" fillId="0" borderId="277" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="358" fillId="0" borderId="278" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="359" fillId="0" borderId="279" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="360" fillId="0" borderId="280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="361" fillId="0" borderId="281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="362" fillId="0" borderId="282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="363" fillId="0" borderId="283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="364" fillId="0" borderId="284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="365" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="366" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="368" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="370" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="372" fillId="0" borderId="289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="373" fillId="0" borderId="290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="374" fillId="0" borderId="291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="375" fillId="0" borderId="292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="376" fillId="0" borderId="293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="377" fillId="0" borderId="294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="378" fillId="0" borderId="295" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="379" fillId="0" borderId="296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="380" fillId="0" borderId="297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="381" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="382" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="383" fillId="0" borderId="300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="384" fillId="0" borderId="301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="385" fillId="0" borderId="302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="386" fillId="0" borderId="303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="387" fillId="0" borderId="304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="388" fillId="0" borderId="305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="389" fillId="0" borderId="306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="390" fillId="0" borderId="307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="391" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="392" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="393" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="394" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="395" fillId="0" borderId="312" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="396" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="397" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="398" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="399" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="401" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="403" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="405" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="407" fillId="0" borderId="320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="409" fillId="0" borderId="321" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="411" fillId="0" borderId="322" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="413" fillId="0" borderId="323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="415" fillId="0" borderId="324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="416" fillId="0" borderId="325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="417" fillId="0" borderId="326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="418" fillId="0" borderId="327" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="419" fillId="0" borderId="328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="420" fillId="0" borderId="329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="421" fillId="0" borderId="330" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="422" fillId="0" borderId="331" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="423" fillId="0" borderId="332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="424" fillId="0" borderId="333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="425" fillId="0" borderId="334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="426" fillId="0" borderId="335" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="427" fillId="0" borderId="336" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="428" fillId="0" borderId="337" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="429" fillId="0" borderId="338" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="430" fillId="0" borderId="339" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="431" fillId="0" borderId="340" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="432" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="433" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="434" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="435" fillId="0" borderId="344" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="436" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="437" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="439" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="441" fillId="0" borderId="348" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="443" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="445" fillId="0" borderId="350" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="447" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="449" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="451" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="452" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="453" fillId="0" borderId="355" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="454" fillId="0" borderId="356" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="455" fillId="0" borderId="357" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="456" fillId="0" borderId="358" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="457" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="458" fillId="0" borderId="360" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="459" fillId="0" borderId="361" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="460" fillId="0" borderId="362" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="461" fillId="0" borderId="363" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="462" fillId="0" borderId="364" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="463" fillId="0" borderId="365" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="464" fillId="0" borderId="366" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="465" fillId="0" borderId="367" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="466" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="467" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="468" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="469" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="470" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="471" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="472" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="473" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="474" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="475" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="476" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="477" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="478" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="479" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="480" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="481" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="482" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="483" fillId="0" borderId="385" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="484" fillId="0" borderId="386" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="485" fillId="0" borderId="387" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="486" fillId="0" borderId="388" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="487" fillId="0" borderId="389" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="488" fillId="0" borderId="390" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="489" fillId="0" borderId="391" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="490" fillId="0" borderId="392" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="491" fillId="0" borderId="393" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="492" fillId="0" borderId="394" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="493" fillId="0" borderId="395" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="494" fillId="0" borderId="396" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="495" fillId="0" borderId="397" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="496" fillId="0" borderId="398" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="497" fillId="0" borderId="399" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="498" fillId="0" borderId="400" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="499" fillId="0" borderId="401" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="500" fillId="0" borderId="402" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="501" fillId="0" borderId="403" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="502" fillId="0" borderId="404" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="503" fillId="0" borderId="405" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="504" fillId="0" borderId="406" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="505" fillId="0" borderId="407" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="506" fillId="0" borderId="408" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="507" fillId="0" borderId="409" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="508" fillId="0" borderId="410" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="509" fillId="0" borderId="411" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="510" fillId="0" borderId="412" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="511" fillId="0" borderId="413" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="512" fillId="0" borderId="414" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="513" fillId="0" borderId="415" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="514" fillId="0" borderId="416" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="515" fillId="0" borderId="417" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="516" fillId="0" borderId="418" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="517" fillId="0" borderId="419" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="518" fillId="0" borderId="420" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="519" fillId="0" borderId="421" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="520" fillId="0" borderId="422" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="521" fillId="0" borderId="423" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="522" fillId="0" borderId="424" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="523" fillId="0" borderId="425" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="524" fillId="0" borderId="426" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="525" fillId="0" borderId="427" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="526" fillId="0" borderId="428" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="527" fillId="0" borderId="429" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="528" fillId="0" borderId="430" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="529" fillId="0" borderId="431" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="530" fillId="0" borderId="432" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="532" fillId="0" borderId="433" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="534" fillId="0" borderId="434" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="536" fillId="0" borderId="435" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="538" fillId="0" borderId="436" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="540" fillId="0" borderId="437" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="542" fillId="0" borderId="438" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="544" fillId="0" borderId="439" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="546" fillId="0" borderId="440" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="548" fillId="0" borderId="441" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="550" fillId="0" borderId="442" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="552" fillId="0" borderId="443" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="554" fillId="0" borderId="444" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="556" fillId="0" borderId="445" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="558" fillId="0" borderId="446" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="560" fillId="0" borderId="447" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="562" fillId="0" borderId="448" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="564" fillId="0" borderId="449" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="566" fillId="0" borderId="450" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="568" fillId="0" borderId="451" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="570" fillId="0" borderId="452" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="572" fillId="0" borderId="453" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="574" fillId="0" borderId="454" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="576" fillId="0" borderId="455" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="578" fillId="0" borderId="456" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="580" fillId="0" borderId="457" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="582" fillId="0" borderId="458" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="584" fillId="0" borderId="459" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="586" fillId="0" borderId="460" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="588" fillId="0" borderId="461" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="590" fillId="0" borderId="462" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="592" fillId="0" borderId="463" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="594" fillId="0" borderId="464" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="596" fillId="0" borderId="465" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="598" fillId="0" borderId="466" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="600" fillId="0" borderId="467" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="602" fillId="0" borderId="468" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="604" fillId="0" borderId="469" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="606" fillId="0" borderId="470" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="608" fillId="0" borderId="471" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="610" fillId="0" borderId="472" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="612" fillId="0" borderId="473" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="614" fillId="0" borderId="474" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="616" fillId="0" borderId="475" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="618" fillId="0" borderId="476" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="620" fillId="0" borderId="477" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="622" fillId="0" borderId="478" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="624" fillId="0" borderId="479" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="626" fillId="0" borderId="480" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="628" fillId="0" borderId="481" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="630" fillId="0" borderId="482" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="632" fillId="0" borderId="483" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="634" fillId="0" borderId="484" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="636" fillId="0" borderId="485" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="638" fillId="0" borderId="486" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="640" fillId="0" borderId="487" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="642" fillId="0" borderId="488" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="644" fillId="0" borderId="489" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="646" fillId="0" borderId="490" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="648" fillId="0" borderId="491" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="650" fillId="0" borderId="492" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="652" fillId="0" borderId="493" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="654" fillId="0" borderId="494" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="656" fillId="0" borderId="495" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="658" fillId="0" borderId="496" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="660" fillId="0" borderId="497" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="662" fillId="0" borderId="498" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="664" fillId="0" borderId="499" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="666" fillId="0" borderId="500" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="668" fillId="0" borderId="501" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="670" fillId="0" borderId="502" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="672" fillId="0" borderId="503" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="674" fillId="0" borderId="504" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4316,246 +8474,246 @@
   <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="31.7109375" style="2" customWidth="true"/>
-    <col min="3" max="3" width="5.11328125" style="3" customWidth="true"/>
-    <col min="6" max="6" width="5.11328125" style="4" customWidth="true"/>
-    <col min="4" max="4" width="11.11328125" style="5" customWidth="true"/>
-    <col min="7" max="7" width="11.11328125" style="6" customWidth="true"/>
-    <col min="5" max="5" width="7.7109375" style="7" customWidth="true"/>
-    <col min="8" max="8" width="7.7109375" style="8" customWidth="true"/>
+    <col min="2" max="2" width="31.7109375" style="254" customWidth="true"/>
+    <col min="3" max="3" width="5.11328125" style="255" customWidth="true"/>
+    <col min="6" max="6" width="5.11328125" style="256" customWidth="true"/>
+    <col min="4" max="4" width="11.11328125" style="257" customWidth="true"/>
+    <col min="7" max="7" width="11.11328125" style="258" customWidth="true"/>
+    <col min="5" max="5" width="7.7109375" style="259" customWidth="true"/>
+    <col min="8" max="8" width="7.7109375" style="260" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="181" t="s">
+    <row r="1" s="253" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="433" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="182" t="s">
+      <c r="B1" s="434" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="183" t="s">
+      <c r="C1" s="435" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="184" t="s">
+      <c r="D1" s="436" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="185" t="s">
+      <c r="E1" s="437" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="186" t="s">
+      <c r="F1" s="438" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="187" t="s">
+      <c r="G1" s="439" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="188" t="s">
+      <c r="H1" s="440" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="189" t="s">
+      <c r="A2" s="441" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="190" t="s">
+      <c r="B2" s="442" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="191" t="s">
+      <c r="C2" s="443" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="192" t="s">
+      <c r="D2" s="444" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="193" t="s">
+      <c r="E2" s="445" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="194" t="s">
+      <c r="F2" s="446" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="195" t="s">
+      <c r="G2" s="447" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="196" t="s">
+      <c r="H2" s="448" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="197" t="s">
+      <c r="A3" s="449" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="198" t="s">
+      <c r="B3" s="450" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="199" t="s">
+      <c r="C3" s="451" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="200" t="s">
+      <c r="D3" s="452" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="201" t="s">
+      <c r="E3" s="453" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="202" t="s">
+      <c r="F3" s="454" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="203" t="s">
+      <c r="G3" s="455" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="204" t="s">
+      <c r="H3" s="456" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="205" t="s">
+      <c r="A4" s="457" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="206" t="s">
+      <c r="B4" s="458" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="207" t="s">
+      <c r="C4" s="459" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="208" t="s">
+      <c r="D4" s="460" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="209" t="s">
+      <c r="E4" s="461" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="210" t="s">
+      <c r="F4" s="462" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="211" t="s">
+      <c r="G4" s="463" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="212" t="s">
+      <c r="H4" s="464" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="213" t="s">
+      <c r="A5" s="465" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="214" t="s">
+      <c r="B5" s="466" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="215" t="s">
+      <c r="C5" s="467" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="216" t="s">
+      <c r="D5" s="468" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="217" t="s">
+      <c r="E5" s="469" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="218" t="s">
+      <c r="F5" s="470" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="219" t="s">
+      <c r="G5" s="471" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="220" t="s">
+      <c r="H5" s="472" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="221" t="s">
+      <c r="A6" s="473" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="222" t="s">
+      <c r="B6" s="474" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="223" t="s">
+      <c r="C6" s="475" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="224" t="s">
+      <c r="D6" s="476" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="225" t="s">
+      <c r="E6" s="477" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="226" t="s">
+      <c r="F6" s="478" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="227" t="s">
+      <c r="G6" s="479" t="s">
         <v>30</v>
       </c>
-      <c r="H6" s="228" t="s">
+      <c r="H6" s="480" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="229" t="s">
+      <c r="A7" s="481" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="230" t="s">
+      <c r="B7" s="482" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="231" t="s">
+      <c r="C7" s="483" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="232" t="s">
+      <c r="D7" s="484" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="233" t="s">
+      <c r="E7" s="485" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="234" t="s">
+      <c r="F7" s="486" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="235" t="s">
+      <c r="G7" s="487" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="236" t="s">
+      <c r="H7" s="488" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="237" t="s">
+      <c r="A8" s="489" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="238" t="s">
+      <c r="B8" s="490" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="239" t="s">
+      <c r="C8" s="491" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="240" t="s">
+      <c r="D8" s="492" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="241" t="s">
+      <c r="E8" s="493" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="242" t="s">
+      <c r="F8" s="494" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="243" t="s">
+      <c r="G8" s="495" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="244" t="s">
+      <c r="H8" s="496" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="245" t="s">
+      <c r="A9" s="497" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="246" t="s">
+      <c r="B9" s="498" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="247" t="s">
+      <c r="C9" s="499" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="248" t="s">
+      <c r="D9" s="500" t="s">
         <v>1</v>
       </c>
-      <c r="E9" s="249" t="s">
+      <c r="E9" s="501" t="s">
         <v>1</v>
       </c>
-      <c r="F9" s="250" t="s">
+      <c r="F9" s="502" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="251" t="s">
+      <c r="G9" s="503" t="s">
         <v>1</v>
       </c>
-      <c r="H9" s="252" t="s">
+      <c r="H9" s="504" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>